<commit_message>
feat: execute configured process modules safely
</commit_message>
<xml_diff>
--- a/share/config/orqflow_v0_1/KeySteps.xlsx
+++ b/share/config/orqflow_v0_1/KeySteps.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Document\PyProject\Playwright\OrqFlow_V0.1\share\config\orqflow_v0_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3E9EF3-DDC2-4E60-8355-200572C17332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1CEA4CF-ADAC-4B1E-B628-B2FD63E81C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1020" windowWidth="28800" windowHeight="13395" xr2:uid="{7952E89B-BE15-4916-8DDD-123323AF50EF}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>State</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Application</t>
   </si>
   <si>
-    <t>Moduel</t>
-  </si>
-  <si>
     <t>Common</t>
   </si>
   <si>
@@ -70,6 +67,12 @@
   </si>
   <si>
     <t>LOGIN_APPLICATION</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>image_value_extraction.runtime:run_process</t>
   </si>
 </sst>
 </file>
@@ -141,7 +144,7 @@
     <tableColumn id="3" xr3:uid="{FE310E18-126F-4D27-AA9E-E413F3A7A75A}" name="State"/>
     <tableColumn id="4" xr3:uid="{ACF77BA4-8A99-4B9E-A0BA-168C8A2C04A2}" name="BatchCount"/>
     <tableColumn id="5" xr3:uid="{B78F3D85-461B-4B80-BFA3-F79FAFC468DD}" name="Application"/>
-    <tableColumn id="6" xr3:uid="{E68CFF3F-0A88-4EF6-A5F4-6400A233ACCC}" name="Moduel"/>
+    <tableColumn id="6" xr3:uid="{E68CFF3F-0A88-4EF6-A5F4-6400A233ACCC}" name="Module"/>
     <tableColumn id="7" xr3:uid="{0008BBDB-911A-4FCB-94F9-583EBA908E1F}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -472,7 +475,7 @@
         <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G1" t="s">
         <v>2</v>
@@ -483,13 +486,13 @@
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -497,7 +500,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -505,7 +508,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -513,7 +516,13 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>